<commit_message>
Keep only two sets of tests; improve description fot the tester
</commit_message>
<xml_diff>
--- a/abtesting_instructions/instructions_mvt_1.xlsx
+++ b/abtesting_instructions/instructions_mvt_1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\github\AB-testing-app\abtesting_instructions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B2DB66A-2B56-4C5C-8C44-B52227BE1FE4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C67C8F5-2F78-4B8F-90A0-4A604F6D5857}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-30990" yWindow="2280" windowWidth="25140" windowHeight="17715" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28965" yWindow="4755" windowWidth="28800" windowHeight="11625" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -54,9 +54,6 @@
     <t>Test Condition 3</t>
   </si>
   <si>
-    <t>Test Condition 4</t>
-  </si>
-  <si>
     <t>Test Condition 6</t>
   </si>
   <si>
@@ -64,6 +61,9 @@
   </si>
   <si>
     <t>Low lighting --- Eye blinking: slow anf fast</t>
+  </si>
+  <si>
+    <t>Test Condition 5</t>
   </si>
 </sst>
 </file>
@@ -423,12 +423,12 @@
         <v>8</v>
       </c>
       <c r="B4" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="B5" t="s">
         <v>4</v>
@@ -436,7 +436,7 @@
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="B6" t="s">
         <v>5</v>
@@ -444,10 +444,10 @@
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B7" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
   </sheetData>

</xml_diff>